<commit_message>
Frankie surname in results
</commit_message>
<xml_diff>
--- a/data/leaguedata.xlsx
+++ b/data/leaguedata.xlsx
@@ -227,7 +227,7 @@
     <t xml:space="preserve">October Junior Competition Sixes</t>
   </si>
   <si>
-    <t xml:space="preserve">Frankie</t>
+    <t xml:space="preserve">Frankie Wright</t>
   </si>
   <si>
     <t xml:space="preserve">November 9 Hole</t>
@@ -3417,7 +3417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="51" t="s">
         <v>73</v>
       </c>
@@ -3467,7 +3467,7 @@
       <c r="I78" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J78" s="0"/>
+      <c r="J78" s="13"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="51" t="s">
@@ -3493,7 +3493,7 @@
       <c r="I79" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J79" s="0"/>
+      <c r="J79" s="13"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="51" t="s">
@@ -3519,7 +3519,7 @@
       <c r="I80" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J80" s="0"/>
+      <c r="J80" s="13"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="51" t="s">
@@ -3545,7 +3545,7 @@
       <c r="I81" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J81" s="0"/>
+      <c r="J81" s="13"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="51" t="s">
@@ -3571,7 +3571,7 @@
       <c r="I82" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J82" s="0"/>
+      <c r="J82" s="13"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="51" t="s">
@@ -3597,7 +3597,7 @@
       <c r="I83" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J83" s="0"/>
+      <c r="J83" s="13"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="51" t="s">
@@ -3623,7 +3623,7 @@
       <c r="I84" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J84" s="0"/>
+      <c r="J84" s="13"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="51" t="s">
@@ -3649,7 +3649,7 @@
       <c r="I85" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="J85" s="0"/>
+      <c r="J85" s="13"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="51" t="s">
@@ -3675,7 +3675,7 @@
       <c r="I86" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="J86" s="0"/>
+      <c r="J86" s="13"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="51" t="s">
@@ -3701,7 +3701,7 @@
       <c r="I87" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="J87" s="0"/>
+      <c r="J87" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I77"/>

</xml_diff>